<commit_message>
slave with new fuses added
</commit_message>
<xml_diff>
--- a/Pre-charge_KR/Pre-charge BOM_smd.xlsx
+++ b/Pre-charge_KR/Pre-charge BOM_smd.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="32">
   <si>
     <t>Pre-charge BOM</t>
   </si>
@@ -35,26 +35,6 @@
   </si>
   <si>
     <t>DNP</t>
-  </si>
-  <si>
-    <t>IC1</t>
-  </si>
-  <si>
-    <t>AL5890-10D-13</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://www.diodes.com/assets/Datasheets/AL5890.pdf</t>
-    </r>
-  </si>
-  <si>
-    <t>AL589010D13:AL589010D13</t>
   </si>
   <si>
     <t>IC2</t>
@@ -77,10 +57,10 @@
     <t>TLV1701AIDBVT:SOT95P280X145-5N</t>
   </si>
   <si>
-    <t>U3</t>
-  </si>
-  <si>
-    <t>SN74AHCT1G08DBVR</t>
+    <t>IC3</t>
+  </si>
+  <si>
+    <t>SN74LVC1G11DCKRE4</t>
   </si>
   <si>
     <r>
@@ -90,17 +70,17 @@
         <color indexed="8"/>
         <rFont val="Helvetica Neue"/>
       </rPr>
-      <t>https://www.ti.com/lit/gpn/sn74ahct1g08</t>
+      <t>https://www.ti.com/lit/gpn/sn74lvc1g11</t>
     </r>
   </si>
   <si>
-    <t>Package_TO_SOT_SMD:SOT-23-5</t>
-  </si>
-  <si>
-    <t>U8</t>
-  </si>
-  <si>
-    <t>SN74AHC1G04DBVRE4</t>
+    <t>SOT65:SOT65P210X110-6N</t>
+  </si>
+  <si>
+    <t>IC4</t>
+  </si>
+  <si>
+    <t>SN74LVC1G08IDCKRQ1</t>
   </si>
   <si>
     <r>
@@ -110,14 +90,17 @@
         <color indexed="8"/>
         <rFont val="Helvetica Neue"/>
       </rPr>
-      <t>https://www.ti.com/lit/gpn/sn74ahc1g04</t>
+      <t>https://www.arrow.com/en/products/sn74lvc1g08idckrq1/texas-instruments</t>
     </r>
   </si>
   <si>
-    <t>U10</t>
-  </si>
-  <si>
-    <t>LM7805MPX/NOPB</t>
+    <t>AND:SOT65P210X110-5N</t>
+  </si>
+  <si>
+    <t>Q1,Q3</t>
+  </si>
+  <si>
+    <t>2N7002</t>
   </si>
   <si>
     <r>
@@ -127,11 +110,51 @@
         <color indexed="8"/>
         <rFont val="Helvetica Neue"/>
       </rPr>
-      <t>https://www.ti.com/lit/gpn/lm7800</t>
+      <t>https://www.onsemi.com/pub/Collateral/NDS7002A-D.PDF</t>
     </r>
   </si>
   <si>
-    <t>Package_TO_SOT_SMD:SOT-223-3_TabPin2</t>
+    <t>Package_TO_SOT_SMD:SOT-23</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>MCP1703AT-3302E/MBVAO</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>http://ww1.microchip.com/downloads/en/DeviceDoc/20005122B.pdf</t>
+    </r>
+  </si>
+  <si>
+    <t>Package_TO_SOT_SMD:SOT-89-3</t>
+  </si>
+  <si>
+    <t>U8</t>
+  </si>
+  <si>
+    <t>SN74LVC1G04QDBVRQ1</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://www.ti.com/lit/ds/symlink/sn74lvc1g04-q1.pdf?ts=1769790994920&amp;ref_url=https%253A%252F%252Fwww.ti.com%252Fproduct%252FSN74LVC1G04-Q1%253Futm_source%253Dgoogle%2526utm_medium%253Dcpc%2526utm_campaign%253Dasc-int-null-44700045788370281_prodfolderdynamic-cpc-pf-google-eu_en_int%2526utm_content%253Dprodfolddynamic%2526ds_k%253DDYNAMIC+SEARCH+ADS%2526DCM%253Dyes%2526gclsrc%253Daw.ds%2526gad_source%253D1%2526gad_campaignid%253D19986097158%2526gbraid%253D0AAAAAC068F0fpBCAHRQzdiYR5ZH1pAS9r%2526gclid%253DCj0KCQiAyvHLBhDlARIsAHxl6xpWbozcNXrMhUW4Ae7a2BLoCwemCPV8kKeqLZTtGhXvQCSpkPl4bX4aAha_EALw_wcB</t>
+    </r>
+  </si>
+  <si>
+    <t>Package_TO_SOT_SMD:SOT-23-5</t>
   </si>
 </sst>
 </file>
@@ -1399,14 +1422,14 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:G7"/>
+  <dimension ref="A2:G8"/>
   <sheetFormatPr defaultColWidth="8.33333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="23.8516" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6719" style="1" customWidth="1"/>
-    <col min="3" max="3" width="19.5" style="1" customWidth="1"/>
-    <col min="4" max="4" width="88.8516" style="1" customWidth="1"/>
-    <col min="5" max="5" width="56.1719" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15.8516" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22.3516" style="1" customWidth="1"/>
+    <col min="4" max="4" width="166.672" style="1" customWidth="1"/>
+    <col min="5" max="5" width="82" style="1" customWidth="1"/>
     <col min="6" max="6" width="4.17188" style="1" customWidth="1"/>
     <col min="7" max="7" width="5" style="1" customWidth="1"/>
     <col min="8" max="16384" width="8.35156" style="1" customWidth="1"/>
@@ -1523,44 +1546,66 @@
         <v>22</v>
       </c>
       <c r="E6" t="s" s="11">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F6" s="12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G6" s="13"/>
     </row>
     <row r="7" ht="20.05" customHeight="1">
       <c r="A7" t="s" s="9">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s" s="10">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s" s="11">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s" s="11">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E7" t="s" s="11">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F7" s="12">
         <v>1</v>
       </c>
       <c r="G7" s="13"/>
+    </row>
+    <row r="8" ht="20.05" customHeight="1">
+      <c r="A8" t="s" s="9">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s" s="10">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s" s="11">
+        <v>29</v>
+      </c>
+      <c r="D8" t="s" s="11">
+        <v>30</v>
+      </c>
+      <c r="E8" t="s" s="11">
+        <v>31</v>
+      </c>
+      <c r="F8" s="12">
+        <v>1</v>
+      </c>
+      <c r="G8" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="D3" r:id="rId1" location="" tooltip="" display="https://www.diodes.com/assets/Datasheets/AL5890.pdf"/>
-    <hyperlink ref="D4" r:id="rId2" location="" tooltip="" display="http://www.ti.com/lit/gpn/tlv1701"/>
-    <hyperlink ref="D5" r:id="rId3" location="" tooltip="" display="https://www.ti.com/lit/gpn/sn74ahct1g08"/>
-    <hyperlink ref="D6" r:id="rId4" location="" tooltip="" display="https://www.ti.com/lit/gpn/sn74ahc1g04"/>
-    <hyperlink ref="D7" r:id="rId5" location="" tooltip="" display="https://www.ti.com/lit/gpn/lm7800"/>
+    <hyperlink ref="D3" r:id="rId1" location="" tooltip="" display="http://www.ti.com/lit/gpn/tlv1701"/>
+    <hyperlink ref="D4" r:id="rId2" location="" tooltip="" display="https://www.ti.com/lit/gpn/sn74lvc1g11"/>
+    <hyperlink ref="D5" r:id="rId3" location="" tooltip="" display="https://www.arrow.com/en/products/sn74lvc1g08idckrq1/texas-instruments"/>
+    <hyperlink ref="D6" r:id="rId4" location="" tooltip="" display="https://www.onsemi.com/pub/Collateral/NDS7002A-D.PDF"/>
+    <hyperlink ref="D7" r:id="rId5" location="" tooltip="" display="http://ww1.microchip.com/downloads/en/DeviceDoc/20005122B.pdf"/>
+    <hyperlink ref="D8" r:id="rId6" location="" tooltip="" display="https://www.ti.com/lit/ds/symlink/sn74lvc1g04-q1.pdf?ts=1769790994920&amp;ref_url=https%253A%252F%252Fwww.ti.com%252Fproduct%252FSN74LVC1G04-Q1%253Futm_source%253Dgoogle%2526utm_medium%253Dcpc%2526utm_campaign%253Dasc-int-null-44700045788370281_prodfolderdynamic-cpc-pf-google-eu_en_int%2526utm_content%253Dprodfolddynamic%2526ds_k%253DDYNAMIC+SEARCH+ADS%2526DCM%253Dyes%2526gclsrc%253Daw.ds%2526gad_source%253D1%2526gad_campaignid%253D19986097158%2526gbraid%253D0AAAAAC068F0fpBCAHRQzdiYR5ZH1pAS9r%2526gclid%253DCj0KCQiAyvHLBhDlARIsAHxl6xpWbozcNXrMhUW4Ae7a2BLoCwemCPV8kKeqLZTtGhXvQCSpkPl4bX4aAha_EALw_wcB"/>
   </hyperlinks>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>